<commit_message>
Deepen valuation assumptions, cash-return and terminal checks; add company-specific price hurdles
</commit_message>
<xml_diff>
--- a/model/Equity_Research_Model.xlsx
+++ b/model/Equity_Research_Model.xlsx
@@ -2,14 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2c9c5df39c3f4a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals Sources" sheetId="2" r:id="Ra774eb2600e74280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R3d0f437d121f4f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="4" r:id="R9116deeda2aa45e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Equity Bridge" sheetId="5" r:id="R07f7eca111ea4800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="R47beb28eae5245c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="Rb8c76d79b13843ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PER" sheetId="8" r:id="Rbd00fbe78e044806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd8345f34a1fe444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals Sources" sheetId="2" r:id="R4aedc4f12e9b4598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" r:id="R566be0ed572149a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="4" r:id="R0dcfc6966e194473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Equity Bridge" sheetId="5" r:id="R055876122b8c4ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" r:id="Rfa1c9ccd724849e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="7" r:id="Rc34e75c570ec429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PER" sheetId="8" r:id="Rc0d38d74e11c41e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnostics" sheetId="9" r:id="R1dd5f59f004a4540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Special Cases" sheetId="10" r:id="R35538ae0f3ff44af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -90,7 +92,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -113,6 +115,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -579,7 +584,7 @@
         <x:v>Report version</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>2026-10-18 v2</x:v>
+        <x:v>2026-10-18 v3</x:v>
       </x:c>
       <x:c r="E15" s="4"/>
       <x:c r="F15" s="4"/>
@@ -874,6 +879,1260 @@
       <x:c r="D34" s="4"/>
       <x:c r="E34" s="4"/>
       <x:c r="F34" s="4"/>
+      <x:c r="G34" s="4"/>
+      <x:c r="H34" s="4"/>
+      <x:c r="I34" s="4"/>
+      <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="1"/>
+      <x:c r="B35" s="1"/>
+      <x:c r="C35" s="1"/>
+      <x:c r="D35" s="4"/>
+      <x:c r="E35" s="4"/>
+      <x:c r="F35" s="4"/>
+      <x:c r="G35" s="4"/>
+      <x:c r="H35" s="4"/>
+      <x:c r="I35" s="4"/>
+      <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="1"/>
+      <x:c r="B36" s="1"/>
+      <x:c r="C36" s="1"/>
+      <x:c r="D36" s="4"/>
+      <x:c r="E36" s="4"/>
+      <x:c r="F36" s="4"/>
+      <x:c r="G36" s="4"/>
+      <x:c r="H36" s="4"/>
+      <x:c r="I36" s="4"/>
+      <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="1"/>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="1"/>
+      <x:c r="D37" s="4"/>
+      <x:c r="E37" s="4"/>
+      <x:c r="F37" s="4"/>
+      <x:c r="G37" s="4"/>
+      <x:c r="H37" s="4"/>
+      <x:c r="I37" s="4"/>
+      <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="1"/>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="1"/>
+      <x:c r="D38" s="4"/>
+      <x:c r="E38" s="4"/>
+      <x:c r="F38" s="4"/>
+      <x:c r="G38" s="4"/>
+      <x:c r="H38" s="4"/>
+      <x:c r="I38" s="4"/>
+      <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="1"/>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="1"/>
+      <x:c r="D39" s="4"/>
+      <x:c r="E39" s="4"/>
+      <x:c r="F39" s="4"/>
+      <x:c r="G39" s="4"/>
+      <x:c r="H39" s="4"/>
+      <x:c r="I39" s="4"/>
+      <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="1"/>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="1"/>
+      <x:c r="D40" s="4"/>
+      <x:c r="E40" s="4"/>
+      <x:c r="F40" s="4"/>
+      <x:c r="G40" s="4"/>
+      <x:c r="H40" s="4"/>
+      <x:c r="I40" s="4"/>
+      <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="1"/>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="4"/>
+      <x:c r="E41" s="4"/>
+      <x:c r="F41" s="4"/>
+      <x:c r="G41" s="4"/>
+      <x:c r="H41" s="4"/>
+      <x:c r="I41" s="4"/>
+      <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="1"/>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="1"/>
+      <x:c r="D42" s="4"/>
+      <x:c r="E42" s="4"/>
+      <x:c r="F42" s="4"/>
+      <x:c r="G42" s="4"/>
+      <x:c r="H42" s="4"/>
+      <x:c r="I42" s="4"/>
+      <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="1"/>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="1"/>
+      <x:c r="D43" s="4"/>
+      <x:c r="E43" s="4"/>
+      <x:c r="F43" s="4"/>
+      <x:c r="G43" s="4"/>
+      <x:c r="H43" s="4"/>
+      <x:c r="I43" s="4"/>
+      <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="1"/>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="4"/>
+      <x:c r="E44" s="4"/>
+      <x:c r="F44" s="4"/>
+      <x:c r="G44" s="4"/>
+      <x:c r="H44" s="4"/>
+      <x:c r="I44" s="4"/>
+      <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="1"/>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="1"/>
+      <x:c r="D45" s="4"/>
+      <x:c r="E45" s="4"/>
+      <x:c r="F45" s="4"/>
+      <x:c r="G45" s="4"/>
+      <x:c r="H45" s="4"/>
+      <x:c r="I45" s="4"/>
+      <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="4"/>
+      <x:c r="E46" s="4"/>
+      <x:c r="F46" s="4"/>
+      <x:c r="G46" s="4"/>
+      <x:c r="H46" s="4"/>
+      <x:c r="I46" s="4"/>
+      <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="1"/>
+      <x:c r="B47" s="1"/>
+      <x:c r="C47" s="1"/>
+      <x:c r="D47" s="4"/>
+      <x:c r="E47" s="4"/>
+      <x:c r="F47" s="4"/>
+      <x:c r="G47" s="4"/>
+      <x:c r="H47" s="4"/>
+      <x:c r="I47" s="4"/>
+      <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="1"/>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="1"/>
+      <x:c r="D48" s="4"/>
+      <x:c r="E48" s="4"/>
+      <x:c r="F48" s="4"/>
+      <x:c r="G48" s="4"/>
+      <x:c r="H48" s="4"/>
+      <x:c r="I48" s="4"/>
+      <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="1"/>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="1"/>
+      <x:c r="D49" s="4"/>
+      <x:c r="E49" s="4"/>
+      <x:c r="F49" s="4"/>
+      <x:c r="G49" s="4"/>
+      <x:c r="H49" s="4"/>
+      <x:c r="I49" s="4"/>
+      <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="1"/>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="1"/>
+      <x:c r="D50" s="4"/>
+      <x:c r="E50" s="4"/>
+      <x:c r="F50" s="4"/>
+      <x:c r="G50" s="4"/>
+      <x:c r="H50" s="4"/>
+      <x:c r="I50" s="4"/>
+      <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="1"/>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="1"/>
+      <x:c r="D51" s="4"/>
+      <x:c r="E51" s="4"/>
+      <x:c r="F51" s="4"/>
+      <x:c r="G51" s="4"/>
+      <x:c r="H51" s="4"/>
+      <x:c r="I51" s="4"/>
+      <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="1"/>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="1"/>
+      <x:c r="D52" s="4"/>
+      <x:c r="E52" s="4"/>
+      <x:c r="F52" s="4"/>
+      <x:c r="G52" s="4"/>
+      <x:c r="H52" s="4"/>
+      <x:c r="I52" s="4"/>
+      <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="1"/>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="1"/>
+      <x:c r="D53" s="4"/>
+      <x:c r="E53" s="4"/>
+      <x:c r="F53" s="4"/>
+      <x:c r="G53" s="4"/>
+      <x:c r="H53" s="4"/>
+      <x:c r="I53" s="4"/>
+      <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="4"/>
+      <x:c r="E54" s="4"/>
+      <x:c r="F54" s="4"/>
+      <x:c r="G54" s="4"/>
+      <x:c r="H54" s="4"/>
+      <x:c r="I54" s="4"/>
+      <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="4"/>
+      <x:c r="E55" s="4"/>
+      <x:c r="F55" s="4"/>
+      <x:c r="G55" s="4"/>
+      <x:c r="H55" s="4"/>
+      <x:c r="I55" s="4"/>
+      <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="4"/>
+      <x:c r="E56" s="4"/>
+      <x:c r="F56" s="4"/>
+      <x:c r="G56" s="4"/>
+      <x:c r="H56" s="4"/>
+      <x:c r="I56" s="4"/>
+      <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="1"/>
+      <x:c r="B57" s="1"/>
+      <x:c r="C57" s="1"/>
+      <x:c r="D57" s="4"/>
+      <x:c r="E57" s="4"/>
+      <x:c r="F57" s="4"/>
+      <x:c r="G57" s="4"/>
+      <x:c r="H57" s="4"/>
+      <x:c r="I57" s="4"/>
+      <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="1"/>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="1"/>
+      <x:c r="D58" s="4"/>
+      <x:c r="E58" s="4"/>
+      <x:c r="F58" s="4"/>
+      <x:c r="G58" s="4"/>
+      <x:c r="H58" s="4"/>
+      <x:c r="I58" s="4"/>
+      <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="1"/>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="1"/>
+      <x:c r="D59" s="4"/>
+      <x:c r="E59" s="4"/>
+      <x:c r="F59" s="4"/>
+      <x:c r="G59" s="4"/>
+      <x:c r="H59" s="4"/>
+      <x:c r="I59" s="4"/>
+      <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="1"/>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="1"/>
+      <x:c r="D60" s="4"/>
+      <x:c r="E60" s="4"/>
+      <x:c r="F60" s="4"/>
+      <x:c r="G60" s="4"/>
+      <x:c r="H60" s="4"/>
+      <x:c r="I60" s="4"/>
+      <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="1"/>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="1"/>
+      <x:c r="D61" s="4"/>
+      <x:c r="E61" s="4"/>
+      <x:c r="F61" s="4"/>
+      <x:c r="G61" s="4"/>
+      <x:c r="H61" s="4"/>
+      <x:c r="I61" s="4"/>
+      <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="1"/>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="1"/>
+      <x:c r="D62" s="4"/>
+      <x:c r="E62" s="4"/>
+      <x:c r="F62" s="4"/>
+      <x:c r="G62" s="4"/>
+      <x:c r="H62" s="4"/>
+      <x:c r="I62" s="4"/>
+      <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="1"/>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="1"/>
+      <x:c r="D63" s="4"/>
+      <x:c r="E63" s="4"/>
+      <x:c r="F63" s="4"/>
+      <x:c r="G63" s="4"/>
+      <x:c r="H63" s="4"/>
+      <x:c r="I63" s="4"/>
+      <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="1"/>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="1"/>
+      <x:c r="D64" s="4"/>
+      <x:c r="E64" s="4"/>
+      <x:c r="F64" s="4"/>
+      <x:c r="G64" s="4"/>
+      <x:c r="H64" s="4"/>
+      <x:c r="I64" s="4"/>
+      <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="1"/>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="1"/>
+      <x:c r="D65" s="4"/>
+      <x:c r="E65" s="4"/>
+      <x:c r="F65" s="4"/>
+      <x:c r="G65" s="4"/>
+      <x:c r="H65" s="4"/>
+      <x:c r="I65" s="4"/>
+      <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="22" customHeight="1">
+      <x:c r="A66" s="1"/>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="1"/>
+      <x:c r="D66" s="4"/>
+      <x:c r="E66" s="4"/>
+      <x:c r="F66" s="4"/>
+      <x:c r="G66" s="4"/>
+      <x:c r="H66" s="4"/>
+      <x:c r="I66" s="4"/>
+      <x:c r="J66" s="1"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="22" customHeight="1">
+      <x:c r="A67" s="1"/>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="1"/>
+      <x:c r="D67" s="4"/>
+      <x:c r="E67" s="4"/>
+      <x:c r="F67" s="4"/>
+      <x:c r="G67" s="4"/>
+      <x:c r="H67" s="4"/>
+      <x:c r="I67" s="4"/>
+      <x:c r="J67" s="1"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="22" customHeight="1">
+      <x:c r="A68" s="1"/>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="4"/>
+      <x:c r="E68" s="4"/>
+      <x:c r="F68" s="4"/>
+      <x:c r="G68" s="4"/>
+      <x:c r="H68" s="4"/>
+      <x:c r="I68" s="4"/>
+      <x:c r="J68" s="1"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="22" customHeight="1">
+      <x:c r="A69" s="1"/>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="4"/>
+      <x:c r="E69" s="4"/>
+      <x:c r="F69" s="4"/>
+      <x:c r="G69" s="4"/>
+      <x:c r="H69" s="4"/>
+      <x:c r="I69" s="4"/>
+      <x:c r="J69" s="1"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="22" customHeight="1">
+      <x:c r="A70" s="1"/>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="4"/>
+      <x:c r="E70" s="4"/>
+      <x:c r="F70" s="4"/>
+      <x:c r="G70" s="4"/>
+      <x:c r="H70" s="4"/>
+      <x:c r="I70" s="4"/>
+      <x:c r="J70" s="1"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="1"/>
+    </x:row>
+    <x:row r="71" ht="22" customHeight="1">
+      <x:c r="A71" s="1"/>
+      <x:c r="B71" s="1"/>
+      <x:c r="C71" s="1"/>
+      <x:c r="D71" s="4"/>
+      <x:c r="E71" s="4"/>
+      <x:c r="F71" s="4"/>
+      <x:c r="G71" s="4"/>
+      <x:c r="H71" s="4"/>
+      <x:c r="I71" s="4"/>
+      <x:c r="J71" s="1"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="1"/>
+    </x:row>
+    <x:row r="72" ht="22" customHeight="1">
+      <x:c r="A72" s="1"/>
+      <x:c r="B72" s="1"/>
+      <x:c r="C72" s="1"/>
+      <x:c r="D72" s="4"/>
+      <x:c r="E72" s="4"/>
+      <x:c r="F72" s="4"/>
+      <x:c r="G72" s="4"/>
+      <x:c r="H72" s="4"/>
+      <x:c r="I72" s="4"/>
+      <x:c r="J72" s="1"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="1"/>
+    </x:row>
+    <x:row r="73" ht="22" customHeight="1">
+      <x:c r="A73" s="1"/>
+      <x:c r="B73" s="1"/>
+      <x:c r="C73" s="1"/>
+      <x:c r="D73" s="4"/>
+      <x:c r="E73" s="4"/>
+      <x:c r="F73" s="4"/>
+      <x:c r="G73" s="4"/>
+      <x:c r="H73" s="4"/>
+      <x:c r="I73" s="4"/>
+      <x:c r="J73" s="1"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="1"/>
+    </x:row>
+    <x:row r="74" ht="22" customHeight="1">
+      <x:c r="A74" s="1"/>
+      <x:c r="B74" s="1"/>
+      <x:c r="C74" s="1"/>
+      <x:c r="D74" s="4"/>
+      <x:c r="E74" s="4"/>
+      <x:c r="F74" s="4"/>
+      <x:c r="G74" s="4"/>
+      <x:c r="H74" s="4"/>
+      <x:c r="I74" s="4"/>
+      <x:c r="J74" s="1"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="1"/>
+    </x:row>
+    <x:row r="75" ht="22" customHeight="1">
+      <x:c r="A75" s="1"/>
+      <x:c r="B75" s="1"/>
+      <x:c r="C75" s="1"/>
+      <x:c r="D75" s="4"/>
+      <x:c r="E75" s="4"/>
+      <x:c r="F75" s="4"/>
+      <x:c r="G75" s="4"/>
+      <x:c r="H75" s="4"/>
+      <x:c r="I75" s="4"/>
+      <x:c r="J75" s="1"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="1"/>
+    </x:row>
+    <x:row r="76" ht="22" customHeight="1">
+      <x:c r="A76" s="1"/>
+      <x:c r="B76" s="1"/>
+      <x:c r="C76" s="1"/>
+      <x:c r="D76" s="4"/>
+      <x:c r="E76" s="4"/>
+      <x:c r="F76" s="4"/>
+      <x:c r="G76" s="4"/>
+      <x:c r="H76" s="4"/>
+      <x:c r="I76" s="4"/>
+      <x:c r="J76" s="1"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="1"/>
+    </x:row>
+    <x:row r="77" ht="22" customHeight="1">
+      <x:c r="A77" s="1"/>
+      <x:c r="B77" s="1"/>
+      <x:c r="C77" s="1"/>
+      <x:c r="D77" s="4"/>
+      <x:c r="E77" s="4"/>
+      <x:c r="F77" s="4"/>
+      <x:c r="G77" s="4"/>
+      <x:c r="H77" s="4"/>
+      <x:c r="I77" s="4"/>
+      <x:c r="J77" s="1"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="1"/>
+    </x:row>
+    <x:row r="78" ht="22" customHeight="1">
+      <x:c r="A78" s="1"/>
+      <x:c r="B78" s="1"/>
+      <x:c r="C78" s="1"/>
+      <x:c r="D78" s="4"/>
+      <x:c r="E78" s="4"/>
+      <x:c r="F78" s="4"/>
+      <x:c r="G78" s="4"/>
+      <x:c r="H78" s="4"/>
+      <x:c r="I78" s="4"/>
+      <x:c r="J78" s="1"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="1"/>
+    </x:row>
+    <x:row r="79" ht="22" customHeight="1">
+      <x:c r="A79" s="1"/>
+      <x:c r="B79" s="1"/>
+      <x:c r="C79" s="1"/>
+      <x:c r="D79" s="4"/>
+      <x:c r="E79" s="4"/>
+      <x:c r="F79" s="4"/>
+      <x:c r="G79" s="4"/>
+      <x:c r="H79" s="4"/>
+      <x:c r="I79" s="4"/>
+      <x:c r="J79" s="1"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="1"/>
+    </x:row>
+    <x:row r="80" ht="22" customHeight="1">
+      <x:c r="A80" s="1"/>
+      <x:c r="B80" s="1"/>
+      <x:c r="C80" s="1"/>
+      <x:c r="D80" s="4"/>
+      <x:c r="E80" s="4"/>
+      <x:c r="F80" s="4"/>
+      <x:c r="G80" s="4"/>
+      <x:c r="H80" s="4"/>
+      <x:c r="I80" s="4"/>
+      <x:c r="J80" s="1"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="1"/>
+    </x:row>
+    <x:row r="81" ht="22" customHeight="1">
+      <x:c r="A81" s="1"/>
+      <x:c r="B81" s="1"/>
+      <x:c r="C81" s="1"/>
+      <x:c r="D81" s="1"/>
+      <x:c r="E81" s="1"/>
+      <x:c r="F81" s="1"/>
+      <x:c r="G81" s="1"/>
+      <x:c r="H81" s="1"/>
+      <x:c r="I81" s="1"/>
+      <x:c r="J81" s="1"/>
+      <x:c r="K81" s="1"/>
+      <x:c r="L81" s="1"/>
+    </x:row>
+    <x:row r="82" ht="22" customHeight="1">
+      <x:c r="A82" s="1"/>
+      <x:c r="B82" s="1"/>
+      <x:c r="C82" s="1"/>
+      <x:c r="D82" s="1"/>
+      <x:c r="E82" s="1"/>
+      <x:c r="F82" s="1"/>
+      <x:c r="G82" s="1"/>
+      <x:c r="H82" s="1"/>
+      <x:c r="I82" s="1"/>
+      <x:c r="J82" s="1"/>
+      <x:c r="K82" s="1"/>
+      <x:c r="L82" s="1"/>
+    </x:row>
+    <x:row r="83" ht="22" customHeight="1">
+      <x:c r="A83" s="1"/>
+      <x:c r="B83" s="1"/>
+      <x:c r="C83" s="1"/>
+      <x:c r="D83" s="1"/>
+      <x:c r="E83" s="1"/>
+      <x:c r="F83" s="1"/>
+      <x:c r="G83" s="1"/>
+      <x:c r="H83" s="1"/>
+      <x:c r="I83" s="1"/>
+      <x:c r="J83" s="1"/>
+      <x:c r="K83" s="1"/>
+      <x:c r="L83" s="1"/>
+    </x:row>
+    <x:row r="84" ht="22" customHeight="1">
+      <x:c r="A84" s="1"/>
+      <x:c r="B84" s="1"/>
+      <x:c r="C84" s="1"/>
+      <x:c r="D84" s="1"/>
+      <x:c r="E84" s="1"/>
+      <x:c r="F84" s="1"/>
+      <x:c r="G84" s="1"/>
+      <x:c r="H84" s="1"/>
+      <x:c r="I84" s="1"/>
+      <x:c r="J84" s="1"/>
+      <x:c r="K84" s="1"/>
+      <x:c r="L84" s="1"/>
+    </x:row>
+    <x:row r="85" ht="22" customHeight="1">
+      <x:c r="A85" s="1"/>
+      <x:c r="B85" s="1"/>
+      <x:c r="C85" s="1"/>
+      <x:c r="D85" s="1"/>
+      <x:c r="E85" s="1"/>
+      <x:c r="F85" s="1"/>
+      <x:c r="G85" s="1"/>
+      <x:c r="H85" s="1"/>
+      <x:c r="I85" s="1"/>
+      <x:c r="J85" s="1"/>
+      <x:c r="K85" s="1"/>
+      <x:c r="L85" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="65" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="2" t="str">
+        <x:v>Special Cases</x:v>
+      </x:c>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="1"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Case selected</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="str">
+        <x:f>Inputs!D3</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="1"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="1"/>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
+      <x:c r="G6" s="1"/>
+      <x:c r="H6" s="1"/>
+      <x:c r="I6" s="1"/>
+      <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="1"/>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="16" t="str">
+        <x:v>Economic assumption review</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>Active case</x:v>
+      </x:c>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
+      <x:c r="G7" s="1"/>
+      <x:c r="H7" s="1"/>
+      <x:c r="I7" s="1"/>
+      <x:c r="J7" s="1"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="29" customHeight="1">
+      <x:c r="A8" s="1"/>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1" t="str">
+        <x:v>DCF: remaining EB exchanged</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="n">
+        <x:f>(DCF!D24+Inputs!$D$62)*1000/(DCF!D25+Inputs!$D$63)</x:f>
+        <x:v>26457.04636997145</x:v>
+      </x:c>
+      <x:c r="E8" s="4"/>
+      <x:c r="F8" s="20" t="str">
+        <x:v>Debt release and economic share count change together.</x:v>
+      </x:c>
+      <x:c r="G8" s="4"/>
+      <x:c r="H8" s="4"/>
+      <x:c r="I8" s="4"/>
+      <x:c r="J8" s="1"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="29" customHeight="1">
+      <x:c r="A9" s="1"/>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1" t="str">
+        <x:v>EUV hurdle: added FCFF in 2032</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="n">
+        <x:f>MAX(Inputs!$D$25*DCF!D25/1000-DCF!D24,0)*(1+Inputs!$D$9)^5*(Inputs!$D$9-Inputs!$D$11)</x:f>
+        <x:v>50.59709993516935</x:v>
+      </x:c>
+      <x:c r="E9" s="4"/>
+      <x:c r="F9" s="20" t="str">
+        <x:v>Added FCFF begins in 2032; earlier contributions = 0.</x:v>
+      </x:c>
+      <x:c r="G9" s="4"/>
+      <x:c r="H9" s="4"/>
+      <x:c r="I9" s="4"/>
+      <x:c r="J9" s="1"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="1"/>
+    </x:row>
+    <x:row r="10" ht="29" customHeight="1">
+      <x:c r="A10" s="1"/>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="1" t="str">
+        <x:v>EUV hurdle: revenue at 20% FCF</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="n">
+        <x:f>D9/Inputs!$D$64</x:f>
+        <x:v>252.9854996758467</x:v>
+      </x:c>
+      <x:c r="E10" s="4"/>
+      <x:c r="F10" s="20" t="str">
+        <x:v>Illustrative FCF margins, not observed EUV economics.</x:v>
+      </x:c>
+      <x:c r="G10" s="4"/>
+      <x:c r="H10" s="4"/>
+      <x:c r="I10" s="4"/>
+      <x:c r="J10" s="1"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="29" customHeight="1">
+      <x:c r="A11" s="1"/>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1" t="str">
+        <x:v>EUV hurdle: revenue at 30% FCF</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="n">
+        <x:f>D9/Inputs!$D$65</x:f>
+        <x:v>168.65699978389782</x:v>
+      </x:c>
+      <x:c r="E11" s="4"/>
+      <x:c r="F11" s="20"/>
+      <x:c r="G11" s="4"/>
+      <x:c r="H11" s="4"/>
+      <x:c r="I11" s="4"/>
+      <x:c r="J11" s="1"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="29" customHeight="1">
+      <x:c r="A12" s="1"/>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="4"/>
+      <x:c r="E12" s="4"/>
+      <x:c r="F12" s="20"/>
+      <x:c r="G12" s="4"/>
+      <x:c r="H12" s="4"/>
+      <x:c r="I12" s="4"/>
+      <x:c r="J12" s="1"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="29" customHeight="1">
+      <x:c r="A13" s="1"/>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1"/>
+      <x:c r="D13" s="4"/>
+      <x:c r="E13" s="4"/>
+      <x:c r="F13" s="20"/>
+      <x:c r="G13" s="4"/>
+      <x:c r="H13" s="4"/>
+      <x:c r="I13" s="4"/>
+      <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="29" customHeight="1">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="4"/>
+      <x:c r="E14" s="4"/>
+      <x:c r="F14" s="20"/>
+      <x:c r="G14" s="4"/>
+      <x:c r="H14" s="4"/>
+      <x:c r="I14" s="4"/>
+      <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="29" customHeight="1">
+      <x:c r="A15" s="1"/>
+      <x:c r="B15" s="1"/>
+      <x:c r="C15" s="1"/>
+      <x:c r="D15" s="4"/>
+      <x:c r="E15" s="4"/>
+      <x:c r="F15" s="20"/>
+      <x:c r="G15" s="4"/>
+      <x:c r="H15" s="4"/>
+      <x:c r="I15" s="4"/>
+      <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="29" customHeight="1">
+      <x:c r="A16" s="1"/>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1" t="str">
+        <x:v>All special cases are local sensitivities, not company guidance.</x:v>
+      </x:c>
+      <x:c r="D16" s="4"/>
+      <x:c r="E16" s="4"/>
+      <x:c r="F16" s="20"/>
+      <x:c r="G16" s="4"/>
+      <x:c r="H16" s="4"/>
+      <x:c r="I16" s="4"/>
+      <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="29" customHeight="1">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="4"/>
+      <x:c r="E17" s="4"/>
+      <x:c r="F17" s="20"/>
+      <x:c r="G17" s="4"/>
+      <x:c r="H17" s="4"/>
+      <x:c r="I17" s="4"/>
+      <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="29" customHeight="1">
+      <x:c r="A18" s="1"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Units: KRW bn / shares mn / prices KRW. See report section 11.</x:v>
+      </x:c>
+      <x:c r="D18" s="4"/>
+      <x:c r="E18" s="4"/>
+      <x:c r="F18" s="20"/>
+      <x:c r="G18" s="4"/>
+      <x:c r="H18" s="4"/>
+      <x:c r="I18" s="4"/>
+      <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="29" customHeight="1">
+      <x:c r="A19" s="1"/>
+      <x:c r="B19" s="1"/>
+      <x:c r="C19" s="1"/>
+      <x:c r="D19" s="4"/>
+      <x:c r="E19" s="4"/>
+      <x:c r="F19" s="20"/>
+      <x:c r="G19" s="4"/>
+      <x:c r="H19" s="4"/>
+      <x:c r="I19" s="4"/>
+      <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="29" customHeight="1">
+      <x:c r="A20" s="1"/>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1"/>
+      <x:c r="D20" s="4"/>
+      <x:c r="E20" s="4"/>
+      <x:c r="F20" s="20"/>
+      <x:c r="G20" s="4"/>
+      <x:c r="H20" s="4"/>
+      <x:c r="I20" s="4"/>
+      <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="29" customHeight="1">
+      <x:c r="A21" s="1"/>
+      <x:c r="B21" s="1"/>
+      <x:c r="C21" s="1"/>
+      <x:c r="D21" s="4"/>
+      <x:c r="E21" s="4"/>
+      <x:c r="F21" s="20"/>
+      <x:c r="G21" s="4"/>
+      <x:c r="H21" s="4"/>
+      <x:c r="I21" s="4"/>
+      <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="29" customHeight="1">
+      <x:c r="A22" s="1"/>
+      <x:c r="B22" s="1"/>
+      <x:c r="C22" s="1"/>
+      <x:c r="D22" s="4"/>
+      <x:c r="E22" s="4"/>
+      <x:c r="F22" s="20"/>
+      <x:c r="G22" s="4"/>
+      <x:c r="H22" s="4"/>
+      <x:c r="I22" s="4"/>
+      <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+    </x:row>
+    <x:row r="23" ht="29" customHeight="1">
+      <x:c r="A23" s="1"/>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="4"/>
+      <x:c r="E23" s="4"/>
+      <x:c r="F23" s="20"/>
+      <x:c r="G23" s="4"/>
+      <x:c r="H23" s="4"/>
+      <x:c r="I23" s="4"/>
+      <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="29" customHeight="1">
+      <x:c r="A24" s="1"/>
+      <x:c r="B24" s="1"/>
+      <x:c r="C24" s="1"/>
+      <x:c r="D24" s="4"/>
+      <x:c r="E24" s="4"/>
+      <x:c r="F24" s="20"/>
+      <x:c r="G24" s="4"/>
+      <x:c r="H24" s="4"/>
+      <x:c r="I24" s="4"/>
+      <x:c r="J24" s="1"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1"/>
+    </x:row>
+    <x:row r="25" ht="29" customHeight="1">
+      <x:c r="A25" s="1"/>
+      <x:c r="B25" s="1"/>
+      <x:c r="C25" s="1"/>
+      <x:c r="D25" s="4"/>
+      <x:c r="E25" s="4"/>
+      <x:c r="F25" s="20"/>
+      <x:c r="G25" s="4"/>
+      <x:c r="H25" s="4"/>
+      <x:c r="I25" s="4"/>
+      <x:c r="J25" s="1"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1"/>
+    </x:row>
+    <x:row r="26" ht="29" customHeight="1">
+      <x:c r="A26" s="1"/>
+      <x:c r="B26" s="1"/>
+      <x:c r="C26" s="1"/>
+      <x:c r="D26" s="4"/>
+      <x:c r="E26" s="4"/>
+      <x:c r="F26" s="20"/>
+      <x:c r="G26" s="4"/>
+      <x:c r="H26" s="4"/>
+      <x:c r="I26" s="4"/>
+      <x:c r="J26" s="1"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1"/>
+    </x:row>
+    <x:row r="27" ht="29" customHeight="1">
+      <x:c r="A27" s="1"/>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="4"/>
+      <x:c r="E27" s="4"/>
+      <x:c r="F27" s="20"/>
+      <x:c r="G27" s="4"/>
+      <x:c r="H27" s="4"/>
+      <x:c r="I27" s="4"/>
+      <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+    </x:row>
+    <x:row r="28" ht="29" customHeight="1">
+      <x:c r="A28" s="1"/>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="4"/>
+      <x:c r="E28" s="4"/>
+      <x:c r="F28" s="20"/>
+      <x:c r="G28" s="4"/>
+      <x:c r="H28" s="4"/>
+      <x:c r="I28" s="4"/>
+      <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+    </x:row>
+    <x:row r="29" ht="29" customHeight="1">
+      <x:c r="A29" s="1"/>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="4"/>
+      <x:c r="E29" s="4"/>
+      <x:c r="F29" s="20"/>
+      <x:c r="G29" s="4"/>
+      <x:c r="H29" s="4"/>
+      <x:c r="I29" s="4"/>
+      <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+    </x:row>
+    <x:row r="30" ht="29" customHeight="1">
+      <x:c r="A30" s="1"/>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="4"/>
+      <x:c r="E30" s="4"/>
+      <x:c r="F30" s="20"/>
+      <x:c r="G30" s="4"/>
+      <x:c r="H30" s="4"/>
+      <x:c r="I30" s="4"/>
+      <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+    </x:row>
+    <x:row r="31" ht="29" customHeight="1">
+      <x:c r="A31" s="1"/>
+      <x:c r="B31" s="1"/>
+      <x:c r="C31" s="1"/>
+      <x:c r="D31" s="4"/>
+      <x:c r="E31" s="4"/>
+      <x:c r="F31" s="20"/>
+      <x:c r="G31" s="4"/>
+      <x:c r="H31" s="4"/>
+      <x:c r="I31" s="4"/>
+      <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+    </x:row>
+    <x:row r="32" ht="29" customHeight="1">
+      <x:c r="A32" s="1"/>
+      <x:c r="B32" s="1"/>
+      <x:c r="C32" s="1"/>
+      <x:c r="D32" s="4"/>
+      <x:c r="E32" s="4"/>
+      <x:c r="F32" s="20"/>
+      <x:c r="G32" s="4"/>
+      <x:c r="H32" s="4"/>
+      <x:c r="I32" s="4"/>
+      <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+    </x:row>
+    <x:row r="33" ht="29" customHeight="1">
+      <x:c r="A33" s="1"/>
+      <x:c r="B33" s="1"/>
+      <x:c r="C33" s="1"/>
+      <x:c r="D33" s="4"/>
+      <x:c r="E33" s="4"/>
+      <x:c r="F33" s="20"/>
+      <x:c r="G33" s="4"/>
+      <x:c r="H33" s="4"/>
+      <x:c r="I33" s="4"/>
+      <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+    </x:row>
+    <x:row r="34" ht="29" customHeight="1">
+      <x:c r="A34" s="1"/>
+      <x:c r="B34" s="1"/>
+      <x:c r="C34" s="1"/>
+      <x:c r="D34" s="4"/>
+      <x:c r="E34" s="4"/>
+      <x:c r="F34" s="20"/>
       <x:c r="G34" s="4"/>
       <x:c r="H34" s="4"/>
       <x:c r="I34" s="4"/>
@@ -4368,7 +5627,9 @@
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="1"/>
       <x:c r="B58" s="1"/>
-      <x:c r="C58" s="1"/>
+      <x:c r="C58" s="1" t="str">
+        <x:v>Review inputs / conditional stresses</x:v>
+      </x:c>
       <x:c r="D58" s="4"/>
       <x:c r="E58" s="4"/>
       <x:c r="F58" s="4"/>
@@ -4396,8 +5657,12 @@
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="1"/>
       <x:c r="B60" s="1"/>
-      <x:c r="C60" s="1"/>
-      <x:c r="D60" s="4"/>
+      <x:c r="C60" s="1" t="str">
+        <x:v>margin_drop</x:v>
+      </x:c>
+      <x:c r="D60" s="6" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
       <x:c r="E60" s="4"/>
       <x:c r="F60" s="4"/>
       <x:c r="G60" s="4"/>
@@ -4410,8 +5675,12 @@
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="1"/>
       <x:c r="B61" s="1"/>
-      <x:c r="C61" s="1"/>
-      <x:c r="D61" s="4"/>
+      <x:c r="C61" s="1" t="str">
+        <x:v>extra_capex</x:v>
+      </x:c>
+      <x:c r="D61" s="6" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
       <x:c r="E61" s="4"/>
       <x:c r="F61" s="4"/>
       <x:c r="G61" s="4"/>
@@ -4424,8 +5693,12 @@
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="1"/>
       <x:c r="B62" s="1"/>
-      <x:c r="C62" s="1"/>
-      <x:c r="D62" s="4"/>
+      <x:c r="C62" s="1" t="str">
+        <x:v>eb_carrying_amount</x:v>
+      </x:c>
+      <x:c r="D62" s="7" t="n">
+        <x:v>13.867513194</x:v>
+      </x:c>
       <x:c r="E62" s="4"/>
       <x:c r="F62" s="4"/>
       <x:c r="G62" s="4"/>
@@ -4438,8 +5711,12 @@
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="1"/>
       <x:c r="B63" s="1"/>
-      <x:c r="C63" s="1"/>
-      <x:c r="D63" s="4"/>
+      <x:c r="C63" s="1" t="str">
+        <x:v>eb_exchange_shares_mn</x:v>
+      </x:c>
+      <x:c r="D63" s="7" t="n">
+        <x:v>0.244504</x:v>
+      </x:c>
       <x:c r="E63" s="4"/>
       <x:c r="F63" s="4"/>
       <x:c r="G63" s="4"/>
@@ -4452,8 +5729,12 @@
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="1"/>
       <x:c r="B64" s="1"/>
-      <x:c r="C64" s="1"/>
-      <x:c r="D64" s="4"/>
+      <x:c r="C64" s="1" t="str">
+        <x:v>euv_fcf_margins_0</x:v>
+      </x:c>
+      <x:c r="D64" s="6" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
       <x:c r="E64" s="4"/>
       <x:c r="F64" s="4"/>
       <x:c r="G64" s="4"/>
@@ -4466,8 +5747,12 @@
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="1"/>
       <x:c r="B65" s="1"/>
-      <x:c r="C65" s="1"/>
-      <x:c r="D65" s="4"/>
+      <x:c r="C65" s="1" t="str">
+        <x:v>euv_fcf_margins_1</x:v>
+      </x:c>
+      <x:c r="D65" s="6" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
       <x:c r="E65" s="4"/>
       <x:c r="F65" s="4"/>
       <x:c r="G65" s="4"/>
@@ -4494,7 +5779,9 @@
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="1"/>
       <x:c r="B67" s="1"/>
-      <x:c r="C67" s="1"/>
+      <x:c r="C67" s="1" t="str">
+        <x:v>Source: research_inputs.json; evidence in report section 06.</x:v>
+      </x:c>
       <x:c r="D67" s="4"/>
       <x:c r="E67" s="4"/>
       <x:c r="F67" s="4"/>
@@ -11845,4 +13132,1371 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="65" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="1"/>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="1"/>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="2" t="str">
+        <x:v>Diagnostics</x:v>
+      </x:c>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="1"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1"/>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Case selected</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="str">
+        <x:f>Inputs!D3</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="1"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="1"/>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
+      <x:c r="G6" s="1"/>
+      <x:c r="H6" s="1"/>
+      <x:c r="I6" s="1"/>
+      <x:c r="J6" s="1"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="1"/>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="16" t="str">
+        <x:v>Economic assumption review</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="str">
+        <x:v>Active case</x:v>
+      </x:c>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
+      <x:c r="G7" s="1"/>
+      <x:c r="H7" s="1"/>
+      <x:c r="I7" s="1"/>
+      <x:c r="J7" s="1"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="29" customHeight="1">
+      <x:c r="A8" s="1"/>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1" t="str">
+        <x:v>2031 reinvestment / NOPAT</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="n">
+        <x:f>(Forecast!I15-Forecast!I14+Forecast!I18)/Forecast!I13</x:f>
+        <x:v>0.11350784282827199</x:v>
+      </x:c>
+      <x:c r="E8" s="4"/>
+      <x:c r="F8" s="20" t="str">
+        <x:v>Conditional stresses; main Base inputs remain selected.</x:v>
+      </x:c>
+      <x:c r="G8" s="4"/>
+      <x:c r="H8" s="4"/>
+      <x:c r="I8" s="4"/>
+      <x:c r="J8" s="1"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="29" customHeight="1">
+      <x:c r="A9" s="1"/>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1" t="str">
+        <x:v>2032 reinvestment / NOPAT</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="n">
+        <x:f>Inputs!$D$11/Inputs!$D$12</x:f>
+        <x:v>0.15384615384615385</x:v>
+      </x:c>
+      <x:c r="E9" s="4"/>
+      <x:c r="F9" s="20"/>
+      <x:c r="G9" s="4"/>
+      <x:c r="H9" s="4"/>
+      <x:c r="I9" s="4"/>
+      <x:c r="J9" s="1"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="1"/>
+    </x:row>
+    <x:row r="10" ht="29" customHeight="1">
+      <x:c r="A10" s="1"/>
+      <x:c r="B10" s="1"/>
+      <x:c r="C10" s="1" t="str">
+        <x:v>FCFF 2032 / 2031 - 1</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:f>DCF!D17/Forecast!I19-1</x:f>
+        <x:v>-0.026413357304264418</x:v>
+      </x:c>
+      <x:c r="E10" s="4"/>
+      <x:c r="F10" s="20" t="str">
+        <x:v>2032 investment transition can change FCFF discontinuously.</x:v>
+      </x:c>
+      <x:c r="G10" s="4"/>
+      <x:c r="H10" s="4"/>
+      <x:c r="I10" s="4"/>
+      <x:c r="J10" s="1"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="29" customHeight="1">
+      <x:c r="A11" s="1"/>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1" t="str">
+        <x:v>2031 parent ROE</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="n">
+        <x:f>RIM!H9/RIM!H8</x:f>
+        <x:v>0.11876639351074555</x:v>
+      </x:c>
+      <x:c r="E11" s="4"/>
+      <x:c r="F11" s="20"/>
+      <x:c r="G11" s="4"/>
+      <x:c r="H11" s="4"/>
+      <x:c r="I11" s="4"/>
+      <x:c r="J11" s="1"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="29" customHeight="1">
+      <x:c r="A12" s="1"/>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1" t="str">
+        <x:v>2032 assumed parent ROE</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="n">
+        <x:f>Inputs!$D$13</x:f>
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="E12" s="4"/>
+      <x:c r="F12" s="20"/>
+      <x:c r="G12" s="4"/>
+      <x:c r="H12" s="4"/>
+      <x:c r="I12" s="4"/>
+      <x:c r="J12" s="1"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="29" customHeight="1">
+      <x:c r="A13" s="1"/>
+      <x:c r="B13" s="1"/>
+      <x:c r="C13" s="1" t="str">
+        <x:v>2031 net cash proxy capped at book</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="n">
+        <x:f>MIN(MAX(Forecast!I26,0),Forecast!I25)</x:f>
+        <x:v>211.60552277793002</x:v>
+      </x:c>
+      <x:c r="E13" s="4"/>
+      <x:c r="F13" s="20" t="str">
+        <x:v>Net cash proxy is not an audited operating-equity split.</x:v>
+      </x:c>
+      <x:c r="G13" s="4"/>
+      <x:c r="H13" s="4"/>
+      <x:c r="I13" s="4"/>
+      <x:c r="J13" s="1"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="29" customHeight="1">
+      <x:c r="A14" s="1"/>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Cash proxy / parent book</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="n">
+        <x:f>D13/Forecast!I25</x:f>
+        <x:v>0.38526499288767546</x:v>
+      </x:c>
+      <x:c r="E14" s="4"/>
+      <x:c r="F14" s="20"/>
+      <x:c r="G14" s="4"/>
+      <x:c r="H14" s="4"/>
+      <x:c r="I14" s="4"/>
+      <x:c r="J14" s="1"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="29" customHeight="1">
+      <x:c r="A15" s="1"/>
+      <x:c r="B15" s="1"/>
+      <x:c r="C15" s="1" t="str">
+        <x:v>Cash split: terminal NI</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="n">
+        <x:f>(Forecast!I25-D13)*Inputs!$D$13+D13*Inputs!$D$20</x:f>
+        <x:v>45.807078342136876</x:v>
+      </x:c>
+      <x:c r="E15" s="4"/>
+      <x:c r="F15" s="20"/>
+      <x:c r="G15" s="4"/>
+      <x:c r="H15" s="4"/>
+      <x:c r="I15" s="4"/>
+      <x:c r="J15" s="1"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="29" customHeight="1">
+      <x:c r="A16" s="1"/>
+      <x:c r="B16" s="1"/>
+      <x:c r="C16" s="1" t="str">
+        <x:v>Cash split: terminal ROE</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="n">
+        <x:f>D15/Forecast!I25</x:f>
+        <x:v>0.08339982567567082</x:v>
+      </x:c>
+      <x:c r="E16" s="4"/>
+      <x:c r="F16" s="20"/>
+      <x:c r="G16" s="4"/>
+      <x:c r="H16" s="4"/>
+      <x:c r="I16" s="4"/>
+      <x:c r="J16" s="1"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="29" customHeight="1">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1" t="str">
+        <x:v>RIM: no terminal excess ROE</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="n">
+        <x:f>(RIM!D18+RIM!D19)*1000/'Cash Equity Bridge'!D23</x:f>
+        <x:v>17720.4357656048</x:v>
+      </x:c>
+      <x:c r="E17" s="4"/>
+      <x:c r="F17" s="20" t="str">
+        <x:v>No excess ROE after the explicit forecast.</x:v>
+      </x:c>
+      <x:c r="G17" s="4"/>
+      <x:c r="H17" s="4"/>
+      <x:c r="I17" s="4"/>
+      <x:c r="J17" s="1"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="29" customHeight="1">
+      <x:c r="A18" s="1"/>
+      <x:c r="B18" s="1"/>
+      <x:c r="C18" s="1" t="str">
+        <x:v>RIM: cash split stress</x:v>
+      </x:c>
+      <x:c r="D18" s="9" t="n">
+        <x:f>(RIM!D18+RIM!D19+(D15-Inputs!$D$10*Forecast!I25)/(Inputs!$D$10-Inputs!$D$11)/(1+Inputs!$D$10)^5)*1000/'Cash Equity Bridge'!D23</x:f>
+        <x:v>13149.432929110973</x:v>
+      </x:c>
+      <x:c r="E18" s="4"/>
+      <x:c r="F18" s="20" t="str">
+        <x:v>Cash yield separated from residual-book ROE.</x:v>
+      </x:c>
+      <x:c r="G18" s="4"/>
+      <x:c r="H18" s="4"/>
+      <x:c r="I18" s="4"/>
+      <x:c r="J18" s="1"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="29" customHeight="1">
+      <x:c r="A19" s="1"/>
+      <x:c r="B19" s="1"/>
+      <x:c r="C19" s="1" t="str">
+        <x:v>DCF: terminal ROIC = WACC</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="n">
+        <x:f>(DCF!D15+DCF!D16/Inputs!$D$9/(1+Inputs!$D$9)^5+DCF!D21+DCF!D22-DCF!D23)*1000/DCF!D25</x:f>
+        <x:v>25402.469630326817</x:v>
+      </x:c>
+      <x:c r="E19" s="4"/>
+      <x:c r="F19" s="20"/>
+      <x:c r="G19" s="4"/>
+      <x:c r="H19" s="4"/>
+      <x:c r="I19" s="4"/>
+      <x:c r="J19" s="1"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="29" customHeight="1">
+      <x:c r="A20" s="1"/>
+      <x:c r="B20" s="1"/>
+      <x:c r="C20" s="1" t="str">
+        <x:v>DCF: excess ROIC value / share</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="n">
+        <x:f>DCF!D26-D19</x:f>
+        <x:v>703.525909740285</x:v>
+      </x:c>
+      <x:c r="E20" s="4"/>
+      <x:c r="F20" s="20"/>
+      <x:c r="G20" s="4"/>
+      <x:c r="H20" s="4"/>
+      <x:c r="I20" s="4"/>
+      <x:c r="J20" s="1"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="29" customHeight="1">
+      <x:c r="A21" s="1"/>
+      <x:c r="B21" s="1"/>
+      <x:c r="C21" s="1" t="str">
+        <x:v>Price hurdle: terminal FCFF bn</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="n">
+        <x:f>(Inputs!$D$25*DCF!D25/1000-DCF!D21-DCF!D22+DCF!D23-DCF!D15)*(1+Inputs!$D$9)^5*(Inputs!$D$9-Inputs!$D$11)</x:f>
+        <x:v>98.55999953231264</x:v>
+      </x:c>
+      <x:c r="E21" s="4"/>
+      <x:c r="F21" s="20" t="str">
+        <x:v>Reference price held unchanged at 2026 year-end.</x:v>
+      </x:c>
+      <x:c r="G21" s="4"/>
+      <x:c r="H21" s="4"/>
+      <x:c r="I21" s="4"/>
+      <x:c r="J21" s="1"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="29" customHeight="1">
+      <x:c r="A22" s="1"/>
+      <x:c r="B22" s="1"/>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Price hurdle: terminal OP margin</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="n">
+        <x:f>D21/(Forecast!I8*(1+Inputs!$D$11)*(1-Inputs!$D$19)*(1-Inputs!$D$11/Inputs!$D$12))</x:f>
+        <x:v>0.4109843248016763</x:v>
+      </x:c>
+      <x:c r="E22" s="4"/>
+      <x:c r="F22" s="20"/>
+      <x:c r="G22" s="4"/>
+      <x:c r="H22" s="4"/>
+      <x:c r="I22" s="4"/>
+      <x:c r="J22" s="1"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1"/>
+    </x:row>
+    <x:row r="23" ht="29" customHeight="1">
+      <x:c r="A23" s="1"/>
+      <x:c r="B23" s="1"/>
+      <x:c r="C23" s="1" t="str">
+        <x:v>Price hurdle: PER normal margin</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="n">
+        <x:f>(Inputs!$D$25/PER!D38*DCF!D25/1000-DCF!D21*Inputs!$D$20)/(Forecast!E8*(1-Inputs!$D$19)*Forecast!E27)</x:f>
+        <x:v>0.42259020953932586</x:v>
+      </x:c>
+      <x:c r="E23" s="4"/>
+      <x:c r="F23" s="20" t="str">
+        <x:v>Theoretical PER is fixed; not empirical peer PER.</x:v>
+      </x:c>
+      <x:c r="G23" s="4"/>
+      <x:c r="H23" s="4"/>
+      <x:c r="I23" s="4"/>
+      <x:c r="J23" s="1"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="29" customHeight="1">
+      <x:c r="A24" s="1"/>
+      <x:c r="B24" s="1"/>
+      <x:c r="C24" s="1" t="str">
+        <x:v>Margin reduction (percentage pts)</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="n">
+        <x:f>Inputs!$D$60</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="E24" s="4"/>
+      <x:c r="F24" s="20"/>
+      <x:c r="G24" s="4"/>
+      <x:c r="H24" s="4"/>
+      <x:c r="I24" s="4"/>
+      <x:c r="J24" s="1"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1"/>
+    </x:row>
+    <x:row r="25" ht="29" customHeight="1">
+      <x:c r="A25" s="1"/>
+      <x:c r="B25" s="1"/>
+      <x:c r="C25" s="1" t="str">
+        <x:v>Additional explicit CAPEX</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="n">
+        <x:f>Inputs!$D$61</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E25" s="4"/>
+      <x:c r="F25" s="20"/>
+      <x:c r="G25" s="4"/>
+      <x:c r="H25" s="4"/>
+      <x:c r="I25" s="4"/>
+      <x:c r="J25" s="1"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1"/>
+    </x:row>
+    <x:row r="26" ht="29" customHeight="1">
+      <x:c r="A26" s="1"/>
+      <x:c r="B26" s="1"/>
+      <x:c r="C26" s="1"/>
+      <x:c r="D26" s="4"/>
+      <x:c r="E26" s="4"/>
+      <x:c r="F26" s="20"/>
+      <x:c r="G26" s="4"/>
+      <x:c r="H26" s="4"/>
+      <x:c r="I26" s="4"/>
+      <x:c r="J26" s="1"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1"/>
+    </x:row>
+    <x:row r="27" ht="29" customHeight="1">
+      <x:c r="A27" s="1"/>
+      <x:c r="B27" s="1"/>
+      <x:c r="C27" s="1" t="str">
+        <x:v>DCF: margin reduction stress</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="n">
+        <x:f>DCF!D26-(Forecast!E8/(1+Inputs!$D$9)^1+Forecast!F8/(1+Inputs!$D$9)^2+Forecast!G8/(1+Inputs!$D$9)^3+Forecast!H8/(1+Inputs!$D$9)^4+Forecast!I8/(1+Inputs!$D$9)^5+Forecast!I8*(1+Inputs!$D$11)*(1-Inputs!$D$11/Inputs!$D$12)/(Inputs!$D$9-Inputs!$D$11)/(1+Inputs!$D$9)^5)*D24*(1-Inputs!$D$19)*1000/DCF!D25</x:f>
+        <x:v>23609.919086163096</x:v>
+      </x:c>
+      <x:c r="E27" s="4"/>
+      <x:c r="F27" s="20"/>
+      <x:c r="G27" s="4"/>
+      <x:c r="H27" s="4"/>
+      <x:c r="I27" s="4"/>
+      <x:c r="J27" s="1"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1"/>
+    </x:row>
+    <x:row r="28" ht="29" customHeight="1">
+      <x:c r="A28" s="1"/>
+      <x:c r="B28" s="1"/>
+      <x:c r="C28" s="1" t="str">
+        <x:v>DCF: additional CAPEX stress</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="n">
+        <x:f>DCF!D26-(Forecast!E15/(1+Inputs!$D$9)^1+Forecast!F15/(1+Inputs!$D$9)^2+Forecast!G15/(1+Inputs!$D$9)^3+Forecast!H15/(1+Inputs!$D$9)^4+Forecast!I15/(1+Inputs!$D$9)^5)*D25*1000/DCF!D25</x:f>
+        <x:v>25089.8246066975</x:v>
+      </x:c>
+      <x:c r="E28" s="4"/>
+      <x:c r="F28" s="20" t="str">
+        <x:v>No benefit to earnings, D&amp;A or terminal from extra CAPEX.</x:v>
+      </x:c>
+      <x:c r="G28" s="4"/>
+      <x:c r="H28" s="4"/>
+      <x:c r="I28" s="4"/>
+      <x:c r="J28" s="1"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1"/>
+    </x:row>
+    <x:row r="29" ht="29" customHeight="1">
+      <x:c r="A29" s="1"/>
+      <x:c r="B29" s="1"/>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="4"/>
+      <x:c r="E29" s="4"/>
+      <x:c r="F29" s="20"/>
+      <x:c r="G29" s="4"/>
+      <x:c r="H29" s="4"/>
+      <x:c r="I29" s="4"/>
+      <x:c r="J29" s="1"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1"/>
+    </x:row>
+    <x:row r="30" ht="29" customHeight="1">
+      <x:c r="A30" s="1"/>
+      <x:c r="B30" s="1"/>
+      <x:c r="C30" s="1" t="str">
+        <x:v>DCF: explicit FCFF / share</x:v>
+      </x:c>
+      <x:c r="D30" s="9" t="n">
+        <x:f>DCF!D15*1000/DCF!D25</x:f>
+        <x:v>6864.427062185699</x:v>
+      </x:c>
+      <x:c r="E30" s="4"/>
+      <x:c r="F30" s="20"/>
+      <x:c r="G30" s="4"/>
+      <x:c r="H30" s="4"/>
+      <x:c r="I30" s="4"/>
+      <x:c r="J30" s="1"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1"/>
+    </x:row>
+    <x:row r="31" ht="29" customHeight="1">
+      <x:c r="A31" s="1"/>
+      <x:c r="B31" s="1"/>
+      <x:c r="C31" s="1" t="str">
+        <x:v>DCF: terminal value / share</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="n">
+        <x:f>DCF!D19*1000/DCF!D25</x:f>
+        <x:v>16251.448515000478</x:v>
+      </x:c>
+      <x:c r="E31" s="4"/>
+      <x:c r="F31" s="20"/>
+      <x:c r="G31" s="4"/>
+      <x:c r="H31" s="4"/>
+      <x:c r="I31" s="4"/>
+      <x:c r="J31" s="1"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1"/>
+    </x:row>
+    <x:row r="32" ht="29" customHeight="1">
+      <x:c r="A32" s="1"/>
+      <x:c r="B32" s="1"/>
+      <x:c r="C32" s="1" t="str">
+        <x:v>DCF: net cash / share</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="n">
+        <x:f>DCF!D21*1000/DCF!D25</x:f>
+        <x:v>3041.356591470648</x:v>
+      </x:c>
+      <x:c r="E32" s="4"/>
+      <x:c r="F32" s="20"/>
+      <x:c r="G32" s="4"/>
+      <x:c r="H32" s="4"/>
+      <x:c r="I32" s="4"/>
+      <x:c r="J32" s="1"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1"/>
+    </x:row>
+    <x:row r="33" ht="29" customHeight="1">
+      <x:c r="A33" s="1"/>
+      <x:c r="B33" s="1"/>
+      <x:c r="C33" s="1" t="str">
+        <x:v>DCF: nonop less NCI / share</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="n">
+        <x:f>(DCF!D22-DCF!D23)*1000/DCF!D25</x:f>
+        <x:v>-51.236628589729904</x:v>
+      </x:c>
+      <x:c r="E33" s="4"/>
+      <x:c r="F33" s="20"/>
+      <x:c r="G33" s="4"/>
+      <x:c r="H33" s="4"/>
+      <x:c r="I33" s="4"/>
+      <x:c r="J33" s="1"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1"/>
+    </x:row>
+    <x:row r="34" ht="29" customHeight="1">
+      <x:c r="A34" s="1"/>
+      <x:c r="B34" s="1"/>
+      <x:c r="C34" s="1" t="str">
+        <x:v>PER: terminal PV / total value</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="n">
+        <x:f>PER!D37/PER!D38</x:f>
+        <x:v>0.7487332560041688</x:v>
+      </x:c>
+      <x:c r="E34" s="4"/>
+      <x:c r="F34" s="20"/>
+      <x:c r="G34" s="4"/>
+      <x:c r="H34" s="4"/>
+      <x:c r="I34" s="4"/>
+      <x:c r="J34" s="1"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="1"/>
+      <x:c r="B35" s="1"/>
+      <x:c r="C35" s="1"/>
+      <x:c r="D35" s="4"/>
+      <x:c r="E35" s="4"/>
+      <x:c r="F35" s="4"/>
+      <x:c r="G35" s="4"/>
+      <x:c r="H35" s="4"/>
+      <x:c r="I35" s="4"/>
+      <x:c r="J35" s="1"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="1"/>
+      <x:c r="B36" s="1"/>
+      <x:c r="C36" s="1"/>
+      <x:c r="D36" s="4"/>
+      <x:c r="E36" s="4"/>
+      <x:c r="F36" s="4"/>
+      <x:c r="G36" s="4"/>
+      <x:c r="H36" s="4"/>
+      <x:c r="I36" s="4"/>
+      <x:c r="J36" s="1"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="1"/>
+      <x:c r="B37" s="1"/>
+      <x:c r="C37" s="1" t="str">
+        <x:v>PER and RIM share DDM assumptions; not independent market evidence.</x:v>
+      </x:c>
+      <x:c r="D37" s="4"/>
+      <x:c r="E37" s="4"/>
+      <x:c r="F37" s="4"/>
+      <x:c r="G37" s="4"/>
+      <x:c r="H37" s="4"/>
+      <x:c r="I37" s="4"/>
+      <x:c r="J37" s="1"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="1"/>
+      <x:c r="B38" s="1"/>
+      <x:c r="C38" s="1"/>
+      <x:c r="D38" s="4"/>
+      <x:c r="E38" s="4"/>
+      <x:c r="F38" s="4"/>
+      <x:c r="G38" s="4"/>
+      <x:c r="H38" s="4"/>
+      <x:c r="I38" s="4"/>
+      <x:c r="J38" s="1"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="1"/>
+      <x:c r="B39" s="1"/>
+      <x:c r="C39" s="1"/>
+      <x:c r="D39" s="4"/>
+      <x:c r="E39" s="4"/>
+      <x:c r="F39" s="4"/>
+      <x:c r="G39" s="4"/>
+      <x:c r="H39" s="4"/>
+      <x:c r="I39" s="4"/>
+      <x:c r="J39" s="1"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="1"/>
+      <x:c r="B40" s="1"/>
+      <x:c r="C40" s="1"/>
+      <x:c r="D40" s="4"/>
+      <x:c r="E40" s="4"/>
+      <x:c r="F40" s="4"/>
+      <x:c r="G40" s="4"/>
+      <x:c r="H40" s="4"/>
+      <x:c r="I40" s="4"/>
+      <x:c r="J40" s="1"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="1"/>
+      <x:c r="B41" s="1"/>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="4"/>
+      <x:c r="E41" s="4"/>
+      <x:c r="F41" s="4"/>
+      <x:c r="G41" s="4"/>
+      <x:c r="H41" s="4"/>
+      <x:c r="I41" s="4"/>
+      <x:c r="J41" s="1"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="1"/>
+      <x:c r="B42" s="1"/>
+      <x:c r="C42" s="1"/>
+      <x:c r="D42" s="4"/>
+      <x:c r="E42" s="4"/>
+      <x:c r="F42" s="4"/>
+      <x:c r="G42" s="4"/>
+      <x:c r="H42" s="4"/>
+      <x:c r="I42" s="4"/>
+      <x:c r="J42" s="1"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="1"/>
+      <x:c r="B43" s="1"/>
+      <x:c r="C43" s="1"/>
+      <x:c r="D43" s="4"/>
+      <x:c r="E43" s="4"/>
+      <x:c r="F43" s="4"/>
+      <x:c r="G43" s="4"/>
+      <x:c r="H43" s="4"/>
+      <x:c r="I43" s="4"/>
+      <x:c r="J43" s="1"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="1"/>
+      <x:c r="B44" s="1"/>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="4"/>
+      <x:c r="E44" s="4"/>
+      <x:c r="F44" s="4"/>
+      <x:c r="G44" s="4"/>
+      <x:c r="H44" s="4"/>
+      <x:c r="I44" s="4"/>
+      <x:c r="J44" s="1"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="1"/>
+      <x:c r="B45" s="1"/>
+      <x:c r="C45" s="1"/>
+      <x:c r="D45" s="4"/>
+      <x:c r="E45" s="4"/>
+      <x:c r="F45" s="4"/>
+      <x:c r="G45" s="4"/>
+      <x:c r="H45" s="4"/>
+      <x:c r="I45" s="4"/>
+      <x:c r="J45" s="1"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="1"/>
+      <x:c r="B46" s="1"/>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="4"/>
+      <x:c r="E46" s="4"/>
+      <x:c r="F46" s="4"/>
+      <x:c r="G46" s="4"/>
+      <x:c r="H46" s="4"/>
+      <x:c r="I46" s="4"/>
+      <x:c r="J46" s="1"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="1"/>
+      <x:c r="B47" s="1"/>
+      <x:c r="C47" s="1"/>
+      <x:c r="D47" s="4"/>
+      <x:c r="E47" s="4"/>
+      <x:c r="F47" s="4"/>
+      <x:c r="G47" s="4"/>
+      <x:c r="H47" s="4"/>
+      <x:c r="I47" s="4"/>
+      <x:c r="J47" s="1"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="1"/>
+      <x:c r="B48" s="1"/>
+      <x:c r="C48" s="1"/>
+      <x:c r="D48" s="4"/>
+      <x:c r="E48" s="4"/>
+      <x:c r="F48" s="4"/>
+      <x:c r="G48" s="4"/>
+      <x:c r="H48" s="4"/>
+      <x:c r="I48" s="4"/>
+      <x:c r="J48" s="1"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="1"/>
+      <x:c r="B49" s="1"/>
+      <x:c r="C49" s="1"/>
+      <x:c r="D49" s="4"/>
+      <x:c r="E49" s="4"/>
+      <x:c r="F49" s="4"/>
+      <x:c r="G49" s="4"/>
+      <x:c r="H49" s="4"/>
+      <x:c r="I49" s="4"/>
+      <x:c r="J49" s="1"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="1"/>
+      <x:c r="B50" s="1"/>
+      <x:c r="C50" s="1"/>
+      <x:c r="D50" s="4"/>
+      <x:c r="E50" s="4"/>
+      <x:c r="F50" s="4"/>
+      <x:c r="G50" s="4"/>
+      <x:c r="H50" s="4"/>
+      <x:c r="I50" s="4"/>
+      <x:c r="J50" s="1"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="1"/>
+      <x:c r="B51" s="1"/>
+      <x:c r="C51" s="1"/>
+      <x:c r="D51" s="4"/>
+      <x:c r="E51" s="4"/>
+      <x:c r="F51" s="4"/>
+      <x:c r="G51" s="4"/>
+      <x:c r="H51" s="4"/>
+      <x:c r="I51" s="4"/>
+      <x:c r="J51" s="1"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="1"/>
+      <x:c r="B52" s="1"/>
+      <x:c r="C52" s="1"/>
+      <x:c r="D52" s="4"/>
+      <x:c r="E52" s="4"/>
+      <x:c r="F52" s="4"/>
+      <x:c r="G52" s="4"/>
+      <x:c r="H52" s="4"/>
+      <x:c r="I52" s="4"/>
+      <x:c r="J52" s="1"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="1"/>
+      <x:c r="B53" s="1"/>
+      <x:c r="C53" s="1"/>
+      <x:c r="D53" s="4"/>
+      <x:c r="E53" s="4"/>
+      <x:c r="F53" s="4"/>
+      <x:c r="G53" s="4"/>
+      <x:c r="H53" s="4"/>
+      <x:c r="I53" s="4"/>
+      <x:c r="J53" s="1"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="1"/>
+      <x:c r="B54" s="1"/>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="4"/>
+      <x:c r="E54" s="4"/>
+      <x:c r="F54" s="4"/>
+      <x:c r="G54" s="4"/>
+      <x:c r="H54" s="4"/>
+      <x:c r="I54" s="4"/>
+      <x:c r="J54" s="1"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="1"/>
+      <x:c r="B55" s="1"/>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="4"/>
+      <x:c r="E55" s="4"/>
+      <x:c r="F55" s="4"/>
+      <x:c r="G55" s="4"/>
+      <x:c r="H55" s="4"/>
+      <x:c r="I55" s="4"/>
+      <x:c r="J55" s="1"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="1"/>
+      <x:c r="B56" s="1"/>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="4"/>
+      <x:c r="E56" s="4"/>
+      <x:c r="F56" s="4"/>
+      <x:c r="G56" s="4"/>
+      <x:c r="H56" s="4"/>
+      <x:c r="I56" s="4"/>
+      <x:c r="J56" s="1"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="1"/>
+      <x:c r="B57" s="1"/>
+      <x:c r="C57" s="1"/>
+      <x:c r="D57" s="4"/>
+      <x:c r="E57" s="4"/>
+      <x:c r="F57" s="4"/>
+      <x:c r="G57" s="4"/>
+      <x:c r="H57" s="4"/>
+      <x:c r="I57" s="4"/>
+      <x:c r="J57" s="1"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="1"/>
+      <x:c r="B58" s="1"/>
+      <x:c r="C58" s="1"/>
+      <x:c r="D58" s="4"/>
+      <x:c r="E58" s="4"/>
+      <x:c r="F58" s="4"/>
+      <x:c r="G58" s="4"/>
+      <x:c r="H58" s="4"/>
+      <x:c r="I58" s="4"/>
+      <x:c r="J58" s="1"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="1"/>
+      <x:c r="B59" s="1"/>
+      <x:c r="C59" s="1"/>
+      <x:c r="D59" s="4"/>
+      <x:c r="E59" s="4"/>
+      <x:c r="F59" s="4"/>
+      <x:c r="G59" s="4"/>
+      <x:c r="H59" s="4"/>
+      <x:c r="I59" s="4"/>
+      <x:c r="J59" s="1"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="1"/>
+      <x:c r="B60" s="1"/>
+      <x:c r="C60" s="1"/>
+      <x:c r="D60" s="4"/>
+      <x:c r="E60" s="4"/>
+      <x:c r="F60" s="4"/>
+      <x:c r="G60" s="4"/>
+      <x:c r="H60" s="4"/>
+      <x:c r="I60" s="4"/>
+      <x:c r="J60" s="1"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="1"/>
+      <x:c r="B61" s="1"/>
+      <x:c r="C61" s="1"/>
+      <x:c r="D61" s="4"/>
+      <x:c r="E61" s="4"/>
+      <x:c r="F61" s="4"/>
+      <x:c r="G61" s="4"/>
+      <x:c r="H61" s="4"/>
+      <x:c r="I61" s="4"/>
+      <x:c r="J61" s="1"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="1"/>
+      <x:c r="B62" s="1"/>
+      <x:c r="C62" s="1"/>
+      <x:c r="D62" s="4"/>
+      <x:c r="E62" s="4"/>
+      <x:c r="F62" s="4"/>
+      <x:c r="G62" s="4"/>
+      <x:c r="H62" s="4"/>
+      <x:c r="I62" s="4"/>
+      <x:c r="J62" s="1"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="1"/>
+      <x:c r="B63" s="1"/>
+      <x:c r="C63" s="1"/>
+      <x:c r="D63" s="4"/>
+      <x:c r="E63" s="4"/>
+      <x:c r="F63" s="4"/>
+      <x:c r="G63" s="4"/>
+      <x:c r="H63" s="4"/>
+      <x:c r="I63" s="4"/>
+      <x:c r="J63" s="1"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="1"/>
+      <x:c r="B64" s="1"/>
+      <x:c r="C64" s="1"/>
+      <x:c r="D64" s="4"/>
+      <x:c r="E64" s="4"/>
+      <x:c r="F64" s="4"/>
+      <x:c r="G64" s="4"/>
+      <x:c r="H64" s="4"/>
+      <x:c r="I64" s="4"/>
+      <x:c r="J64" s="1"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="1"/>
+      <x:c r="B65" s="1"/>
+      <x:c r="C65" s="1"/>
+      <x:c r="D65" s="4"/>
+      <x:c r="E65" s="4"/>
+      <x:c r="F65" s="4"/>
+      <x:c r="G65" s="4"/>
+      <x:c r="H65" s="4"/>
+      <x:c r="I65" s="4"/>
+      <x:c r="J65" s="1"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1"/>
+    </x:row>
+    <x:row r="66" ht="22" customHeight="1">
+      <x:c r="A66" s="1"/>
+      <x:c r="B66" s="1"/>
+      <x:c r="C66" s="1"/>
+      <x:c r="D66" s="4"/>
+      <x:c r="E66" s="4"/>
+      <x:c r="F66" s="4"/>
+      <x:c r="G66" s="4"/>
+      <x:c r="H66" s="4"/>
+      <x:c r="I66" s="4"/>
+      <x:c r="J66" s="1"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="1"/>
+    </x:row>
+    <x:row r="67" ht="22" customHeight="1">
+      <x:c r="A67" s="1"/>
+      <x:c r="B67" s="1"/>
+      <x:c r="C67" s="1"/>
+      <x:c r="D67" s="4"/>
+      <x:c r="E67" s="4"/>
+      <x:c r="F67" s="4"/>
+      <x:c r="G67" s="4"/>
+      <x:c r="H67" s="4"/>
+      <x:c r="I67" s="4"/>
+      <x:c r="J67" s="1"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="1"/>
+    </x:row>
+    <x:row r="68" ht="22" customHeight="1">
+      <x:c r="A68" s="1"/>
+      <x:c r="B68" s="1"/>
+      <x:c r="C68" s="1"/>
+      <x:c r="D68" s="4"/>
+      <x:c r="E68" s="4"/>
+      <x:c r="F68" s="4"/>
+      <x:c r="G68" s="4"/>
+      <x:c r="H68" s="4"/>
+      <x:c r="I68" s="4"/>
+      <x:c r="J68" s="1"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="1"/>
+    </x:row>
+    <x:row r="69" ht="22" customHeight="1">
+      <x:c r="A69" s="1"/>
+      <x:c r="B69" s="1"/>
+      <x:c r="C69" s="1"/>
+      <x:c r="D69" s="4"/>
+      <x:c r="E69" s="4"/>
+      <x:c r="F69" s="4"/>
+      <x:c r="G69" s="4"/>
+      <x:c r="H69" s="4"/>
+      <x:c r="I69" s="4"/>
+      <x:c r="J69" s="1"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="1"/>
+    </x:row>
+    <x:row r="70" ht="22" customHeight="1">
+      <x:c r="A70" s="1"/>
+      <x:c r="B70" s="1"/>
+      <x:c r="C70" s="1"/>
+      <x:c r="D70" s="4"/>
+      <x:c r="E70" s="4"/>
+      <x:c r="F70" s="4"/>
+      <x:c r="G70" s="4"/>
+      <x:c r="H70" s="4"/>
+      <x:c r="I70" s="4"/>
+      <x:c r="J70" s="1"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="1"/>
+    </x:row>
+    <x:row r="71" ht="22" customHeight="1">
+      <x:c r="A71" s="1"/>
+      <x:c r="B71" s="1"/>
+      <x:c r="C71" s="1"/>
+      <x:c r="D71" s="4"/>
+      <x:c r="E71" s="4"/>
+      <x:c r="F71" s="4"/>
+      <x:c r="G71" s="4"/>
+      <x:c r="H71" s="4"/>
+      <x:c r="I71" s="4"/>
+      <x:c r="J71" s="1"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="1"/>
+    </x:row>
+    <x:row r="72" ht="22" customHeight="1">
+      <x:c r="A72" s="1"/>
+      <x:c r="B72" s="1"/>
+      <x:c r="C72" s="1"/>
+      <x:c r="D72" s="4"/>
+      <x:c r="E72" s="4"/>
+      <x:c r="F72" s="4"/>
+      <x:c r="G72" s="4"/>
+      <x:c r="H72" s="4"/>
+      <x:c r="I72" s="4"/>
+      <x:c r="J72" s="1"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="1"/>
+    </x:row>
+    <x:row r="73" ht="22" customHeight="1">
+      <x:c r="A73" s="1"/>
+      <x:c r="B73" s="1"/>
+      <x:c r="C73" s="1"/>
+      <x:c r="D73" s="4"/>
+      <x:c r="E73" s="4"/>
+      <x:c r="F73" s="4"/>
+      <x:c r="G73" s="4"/>
+      <x:c r="H73" s="4"/>
+      <x:c r="I73" s="4"/>
+      <x:c r="J73" s="1"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="1"/>
+    </x:row>
+    <x:row r="74" ht="22" customHeight="1">
+      <x:c r="A74" s="1"/>
+      <x:c r="B74" s="1"/>
+      <x:c r="C74" s="1"/>
+      <x:c r="D74" s="4"/>
+      <x:c r="E74" s="4"/>
+      <x:c r="F74" s="4"/>
+      <x:c r="G74" s="4"/>
+      <x:c r="H74" s="4"/>
+      <x:c r="I74" s="4"/>
+      <x:c r="J74" s="1"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="1"/>
+    </x:row>
+    <x:row r="75" ht="22" customHeight="1">
+      <x:c r="A75" s="1"/>
+      <x:c r="B75" s="1"/>
+      <x:c r="C75" s="1"/>
+      <x:c r="D75" s="4"/>
+      <x:c r="E75" s="4"/>
+      <x:c r="F75" s="4"/>
+      <x:c r="G75" s="4"/>
+      <x:c r="H75" s="4"/>
+      <x:c r="I75" s="4"/>
+      <x:c r="J75" s="1"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="1"/>
+    </x:row>
+    <x:row r="76" ht="22" customHeight="1">
+      <x:c r="A76" s="1"/>
+      <x:c r="B76" s="1"/>
+      <x:c r="C76" s="1"/>
+      <x:c r="D76" s="4"/>
+      <x:c r="E76" s="4"/>
+      <x:c r="F76" s="4"/>
+      <x:c r="G76" s="4"/>
+      <x:c r="H76" s="4"/>
+      <x:c r="I76" s="4"/>
+      <x:c r="J76" s="1"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="1"/>
+    </x:row>
+    <x:row r="77" ht="22" customHeight="1">
+      <x:c r="A77" s="1"/>
+      <x:c r="B77" s="1"/>
+      <x:c r="C77" s="1"/>
+      <x:c r="D77" s="4"/>
+      <x:c r="E77" s="4"/>
+      <x:c r="F77" s="4"/>
+      <x:c r="G77" s="4"/>
+      <x:c r="H77" s="4"/>
+      <x:c r="I77" s="4"/>
+      <x:c r="J77" s="1"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="1"/>
+    </x:row>
+    <x:row r="78" ht="22" customHeight="1">
+      <x:c r="A78" s="1"/>
+      <x:c r="B78" s="1"/>
+      <x:c r="C78" s="1"/>
+      <x:c r="D78" s="4"/>
+      <x:c r="E78" s="4"/>
+      <x:c r="F78" s="4"/>
+      <x:c r="G78" s="4"/>
+      <x:c r="H78" s="4"/>
+      <x:c r="I78" s="4"/>
+      <x:c r="J78" s="1"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="1"/>
+    </x:row>
+    <x:row r="79" ht="22" customHeight="1">
+      <x:c r="A79" s="1"/>
+      <x:c r="B79" s="1"/>
+      <x:c r="C79" s="1"/>
+      <x:c r="D79" s="4"/>
+      <x:c r="E79" s="4"/>
+      <x:c r="F79" s="4"/>
+      <x:c r="G79" s="4"/>
+      <x:c r="H79" s="4"/>
+      <x:c r="I79" s="4"/>
+      <x:c r="J79" s="1"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="1"/>
+    </x:row>
+    <x:row r="80" ht="22" customHeight="1">
+      <x:c r="A80" s="1"/>
+      <x:c r="B80" s="1"/>
+      <x:c r="C80" s="1"/>
+      <x:c r="D80" s="4"/>
+      <x:c r="E80" s="4"/>
+      <x:c r="F80" s="4"/>
+      <x:c r="G80" s="4"/>
+      <x:c r="H80" s="4"/>
+      <x:c r="I80" s="4"/>
+      <x:c r="J80" s="1"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="1"/>
+    </x:row>
+    <x:row r="81" ht="22" customHeight="1">
+      <x:c r="A81" s="1"/>
+      <x:c r="B81" s="1"/>
+      <x:c r="C81" s="1"/>
+      <x:c r="D81" s="1"/>
+      <x:c r="E81" s="1"/>
+      <x:c r="F81" s="1"/>
+      <x:c r="G81" s="1"/>
+      <x:c r="H81" s="1"/>
+      <x:c r="I81" s="1"/>
+      <x:c r="J81" s="1"/>
+      <x:c r="K81" s="1"/>
+      <x:c r="L81" s="1"/>
+    </x:row>
+    <x:row r="82" ht="22" customHeight="1">
+      <x:c r="A82" s="1"/>
+      <x:c r="B82" s="1"/>
+      <x:c r="C82" s="1"/>
+      <x:c r="D82" s="1"/>
+      <x:c r="E82" s="1"/>
+      <x:c r="F82" s="1"/>
+      <x:c r="G82" s="1"/>
+      <x:c r="H82" s="1"/>
+      <x:c r="I82" s="1"/>
+      <x:c r="J82" s="1"/>
+      <x:c r="K82" s="1"/>
+      <x:c r="L82" s="1"/>
+    </x:row>
+    <x:row r="83" ht="22" customHeight="1">
+      <x:c r="A83" s="1"/>
+      <x:c r="B83" s="1"/>
+      <x:c r="C83" s="1"/>
+      <x:c r="D83" s="1"/>
+      <x:c r="E83" s="1"/>
+      <x:c r="F83" s="1"/>
+      <x:c r="G83" s="1"/>
+      <x:c r="H83" s="1"/>
+      <x:c r="I83" s="1"/>
+      <x:c r="J83" s="1"/>
+      <x:c r="K83" s="1"/>
+      <x:c r="L83" s="1"/>
+    </x:row>
+    <x:row r="84" ht="22" customHeight="1">
+      <x:c r="A84" s="1"/>
+      <x:c r="B84" s="1"/>
+      <x:c r="C84" s="1"/>
+      <x:c r="D84" s="1"/>
+      <x:c r="E84" s="1"/>
+      <x:c r="F84" s="1"/>
+      <x:c r="G84" s="1"/>
+      <x:c r="H84" s="1"/>
+      <x:c r="I84" s="1"/>
+      <x:c r="J84" s="1"/>
+      <x:c r="K84" s="1"/>
+      <x:c r="L84" s="1"/>
+    </x:row>
+    <x:row r="85" ht="22" customHeight="1">
+      <x:c r="A85" s="1"/>
+      <x:c r="B85" s="1"/>
+      <x:c r="C85" s="1"/>
+      <x:c r="D85" s="1"/>
+      <x:c r="E85" s="1"/>
+      <x:c r="F85" s="1"/>
+      <x:c r="G85" s="1"/>
+      <x:c r="H85" s="1"/>
+      <x:c r="I85" s="1"/>
+      <x:c r="J85" s="1"/>
+      <x:c r="K85" s="1"/>
+      <x:c r="L85" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>